<commit_message>
re-render: run complete; the morning table and notes
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_johnson_res_solved.xlsx
+++ b/docs/tutorials/files/xslope_johnson_res_solved.xlsx
@@ -8666,17 +8666,17 @@
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A6" s="56" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>shell</v>
       </c>
       <c r="B6" s="57"/>
       <c r="D6" s="56" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>core</v>
       </c>
       <c r="E6" s="57"/>
       <c r="G6" s="56" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
-        <v/>
+        <v>foundation</v>
       </c>
       <c r="H6" s="57"/>
       <c r="J6" s="56" t="str">
@@ -10122,17 +10122,17 @@
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="58" t="str">
         <f>IF(OR(B5="",B5="material"),_xlfn.XLOOKUP(B6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
-        <v/>
+        <v>shell</v>
       </c>
       <c r="B7" s="57"/>
       <c r="D7" s="58" t="str">
         <f>IF(OR(E5="",E5="material"),_xlfn.XLOOKUP(E6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
-        <v/>
+        <v>core</v>
       </c>
       <c r="E7" s="57"/>
       <c r="G7" s="58" t="str">
         <f>IF(OR(H5="",H5="material"),_xlfn.XLOOKUP(H6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
-        <v/>
+        <v>foundation</v>
       </c>
       <c r="H7" s="57"/>
       <c r="J7" s="58" t="str">

</xml_diff>